<commit_message>
Fix trial class name-before-phone flow
</commit_message>
<xml_diff>
--- a/.github/chatbot/leads.xlsx
+++ b/.github/chatbot/leads.xlsx
@@ -694,17 +694,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-02 16:00:19</t>
+          <t>2026-10-02 16:03:57</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Juan Perez (@prueba_full)</t>
+          <t>Carlos Soto (@dup_test)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>8112345678</t>
+          <t>8110001122</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -714,7 +714,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Bosque Santa Anita</t>
+          <t>Guadalupe</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -726,22 +726,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-02 16:03:57</t>
+          <t>2026-10-02 16:04:23</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Carlos Soto (@dup_test)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>8110001122</t>
+          <t>@Pao Maldo</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Running</t>
+          <t>Wellness</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -758,12 +753,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-02 16:04:23</t>
+          <t>2026-10-02 16:05:13</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>@Pao Maldo</t>
+          <t>@Paola</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -785,12 +780,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-02 16:05:13</t>
+          <t>2026-10-02 16:06:34</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>@Paola</t>
+          <t>@Carlos</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -812,17 +807,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-02 16:06:34</t>
+          <t>2026-10-05 13:36:59</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>@Carlos</t>
+          <t>@AnaB00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Wellness</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -839,22 +834,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-05 13:36:59</t>
+          <t>2026-10-05 13:41:14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>@AnaB00</t>
+          <t>@Alexcova</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>HYROX</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Guadalupe</t>
+          <t>Bosque Santa Anita</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -866,17 +861,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-05 13:41:14</t>
+          <t>2026-10-05 13:49:19</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>@Alexcova</t>
+          <t>@branch_test</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>HYROX</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -893,12 +888,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-05 13:49:19</t>
+          <t>2026-10-05 13:49:58</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>@branch_test</t>
+          <t>@DianaTru</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -920,22 +915,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-05 13:49:58</t>
+          <t>2026-10-05 13:50:35</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>@DianaTru</t>
+          <t>@Jurtizz</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>Wellness</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bosque Santa Anita</t>
+          <t>Guadalupe</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -947,22 +942,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-05 13:50:35</t>
+          <t>2026-10-05 13:55:04</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>@Jurtizz</t>
+          <t>@tester</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Wellness</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Guadalupe</t>
+          <t>Sin especificar</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -979,7 +974,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>@tester</t>
+          <t>@ig_12345</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1001,23 +996,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-05 13:55:04</t>
+          <t>2026-10-08 20:50:53</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>@ig_12345</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>Cuanto Cuesta La Mensualidad (@prueba_full)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>8112345678</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>Running</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sin especificar</t>
+          <t>Bosque Santa Anita</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">

</xml_diff>